<commit_message>
fix(board): clarify ferry plan approval progress by discipline
</commit_message>
<xml_diff>
--- a/downloads/ferry-progress-2026-10-02.xlsx
+++ b/downloads/ferry-progress-2026-10-02.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段进度" sheetId="1" r:id="R31aa6eabbb2044b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="专项跟踪" sheetId="2" r:id="R706be5e9714e49dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="3" r:id="R80e233490e5d4a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段进度" sheetId="1" r:id="R6cf28da506f9485b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="专项跟踪" sheetId="2" r:id="R6f03f838ce514f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="3" r:id="Rbc24e8a142e54806"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -43,6 +43,12 @@
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF6B5B35"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FF18334E"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -85,7 +91,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -132,6 +138,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -210,7 +219,23 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Actions" displayName="Actions" ref="A7:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PlanApproval" displayName="PlanApproval" ref="A24:G28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A24:G28"/>
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="船型"/>
+    <x:tableColumn id="2" name="专业"/>
+    <x:tableColumn id="3" name="审批结果"/>
+    <x:tableColumn id="4" name="最新批复日"/>
+    <x:tableColumn id="5" name="已获批批次"/>
+    <x:tableColumn id="6" name="后续落实 / 现场项"/>
+    <x:tableColumn id="7" name="证据ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Actions" displayName="Actions" ref="A7:K23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A7:K23"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
@@ -229,8 +254,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Evidence" displayName="Evidence" ref="A7:F37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Evidence" displayName="Evidence" ref="A7:F37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A7:F37"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="证据ID"/>
@@ -603,21 +628,21 @@
         <x:v>审图</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>多轮获批，全面关闭待核实</x:v>
+        <x:v>电气、轮机主要批次已获批</x:v>
       </x:c>
       <x:c r="C10" s="12" t="d">
         <x:v>2026-09-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
-        <x:v>单层电气答复7月获批；双层电气答复9月获批；两类艉管9月获批。</x:v>
+        <x:v>单层电气答复07-30、修改通知单07-31获A；双层电气答复09-03获A；两类轮机答复07-31、艉管09-02获A。</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
-        <x:v>汇总P项关闭和S/TS现场核查；补船体前窗意见关闭证明。</x:v>
+        <x:v>核准批准图纸清单；S/TS转现场跟踪；船体前窗P项另行核实。</x:v>
       </x:c>
       <x:c r="F10" s="13"/>
       <x:c r="G10" s="14"/>
       <x:c r="H10" s="11" t="str">
-        <x:v>E04、E05、E15、E11、E14、E24</x:v>
+        <x:v>E04、E05、E15、E12、E13、E22、E23、E11、E14；E07、E18、E24</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="82" customHeight="1">
@@ -788,10 +813,165 @@
       <x:c r="G21" s="2"/>
       <x:c r="H21" s="2"/>
     </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="17" t="str">
+        <x:v>审图分船型、分专业进度</x:v>
+      </x:c>
+      <x:c r="B22" s="2"/>
+      <x:c r="C22" s="2"/>
+      <x:c r="D22" s="2"/>
+      <x:c r="E22" s="2"/>
+      <x:c r="F22" s="2"/>
+      <x:c r="G22" s="2"/>
+      <x:c r="H22" s="2"/>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="2"/>
+      <x:c r="B23" s="2"/>
+      <x:c r="C23" s="2"/>
+      <x:c r="D23" s="15" t="str">
+        <x:v>按现有批复记录；全船审批终结待核准批准图纸清单，双层船体前窗P项另行跟踪（E24）。</x:v>
+      </x:c>
+      <x:c r="E23" s="15"/>
+      <x:c r="F23" s="15"/>
+      <x:c r="G23" s="15"/>
+      <x:c r="H23" s="15"/>
+    </x:row>
+    <x:row r="24" ht="36" customHeight="1">
+      <x:c r="A24" s="10" t="str">
+        <x:v>船型</x:v>
+      </x:c>
+      <x:c r="B24" s="10" t="str">
+        <x:v>专业</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>审批结果</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="str">
+        <x:v>最新批复日</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>已获批批次</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="str">
+        <x:v>后续落实 / 现场项</x:v>
+      </x:c>
+      <x:c r="G24" s="10" t="str">
+        <x:v>证据ID</x:v>
+      </x:c>
+      <x:c r="H24" s="2"/>
+    </x:row>
+    <x:row r="25" ht="94" customHeight="1">
+      <x:c r="A25" s="11" t="str">
+        <x:v>单层16</x:v>
+      </x:c>
+      <x:c r="B25" s="11" t="str">
+        <x:v>电气</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="str">
+        <x:v>意见答复及修改获A</x:v>
+      </x:c>
+      <x:c r="D25" s="12" t="d">
+        <x:v>2026-07-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="str">
+        <x:v>004E：003E答复07-30获A；005E：001E修改通知单07-31获A。</x:v>
+      </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>核对批准图纸版本；现场S项单独跟踪。</x:v>
+      </x:c>
+      <x:c r="G25" s="11" t="str">
+        <x:v>E04、E05</x:v>
+      </x:c>
+      <x:c r="H25" s="2"/>
+    </x:row>
+    <x:row r="26" ht="94" customHeight="1">
+      <x:c r="A26" s="11" t="str">
+        <x:v>单层16</x:v>
+      </x:c>
+      <x:c r="B26" s="11" t="str">
+        <x:v>轮机</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="str">
+        <x:v>管系、答复及艉管获A</x:v>
+      </x:c>
+      <x:c r="D26" s="12" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="str">
+        <x:v>006M：B版07-01获A；007M：005M答复07-31获A；008M：艉管09-02获A。</x:v>
+      </x:c>
+      <x:c r="F26" s="11" t="str">
+        <x:v>电机/齿轮箱安装图TS转现场验船师。</x:v>
+      </x:c>
+      <x:c r="G26" s="11" t="str">
+        <x:v>E12、E13、E11；E07</x:v>
+      </x:c>
+      <x:c r="H26" s="2"/>
+    </x:row>
+    <x:row r="27" ht="94" customHeight="1">
+      <x:c r="A27" s="11" t="str">
+        <x:v>双层13、15</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="str">
+        <x:v>电气</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="str">
+        <x:v>001E意见答复获A</x:v>
+      </x:c>
+      <x:c r="D27" s="12" t="d">
+        <x:v>2026-09-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="str">
+        <x:v>002E：001E答复09-03获A。</x:v>
+      </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>核对批准图纸版本；谐波实测等S项单独跟踪。</x:v>
+      </x:c>
+      <x:c r="G27" s="11" t="str">
+        <x:v>E15、E30；E16</x:v>
+      </x:c>
+      <x:c r="H27" s="2"/>
+    </x:row>
+    <x:row r="28" ht="94" customHeight="1">
+      <x:c r="A28" s="11" t="str">
+        <x:v>双层13、15</x:v>
+      </x:c>
+      <x:c r="B28" s="11" t="str">
+        <x:v>轮机</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="str">
+        <x:v>管系、答复及艉管获A</x:v>
+      </x:c>
+      <x:c r="D28" s="12" t="d">
+        <x:v>2026-09-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="str">
+        <x:v>006M：B版07-07获A；007M：005M答复07-31获A；009M：艉管09-02获A。</x:v>
+      </x:c>
+      <x:c r="F28" s="11" t="str">
+        <x:v>电机/齿轮箱安装图TS转现场验船师。</x:v>
+      </x:c>
+      <x:c r="G28" s="11" t="str">
+        <x:v>E22、E23、E14；E18</x:v>
+      </x:c>
+      <x:c r="H28" s="2"/>
+    </x:row>
+    <x:row r="29" ht="30" customHeight="1">
+      <x:c r="A29" s="2"/>
+      <x:c r="B29" s="2"/>
+      <x:c r="C29" s="2"/>
+      <x:c r="D29" s="2"/>
+      <x:c r="E29" s="2"/>
+      <x:c r="F29" s="2"/>
+      <x:c r="G29" s="2"/>
+      <x:c r="H29" s="2"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0517a22812cb4d6c"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb8226c8e9274fe4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a79eef522df427c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1014,7 +1194,7 @@
         <x:v>文件获批</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
-        <x:v>B版管系及005M答复已获A；不代表安装和现场验收完成。</x:v>
+        <x:v>单层B版7月1日、双层B版7月7日获A；两类005M答复7月31日获A。安装和现场验收另行跟踪。</x:v>
       </x:c>
       <x:c r="F10" s="11" t="str">
         <x:v>设计院/船厂</x:v>
@@ -1447,7 +1627,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R987f0c56548b4d0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra051d3b9cb6143e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2164,7 +2344,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re80ba5f546964611"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55a1f1d5791f476b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>